<commit_message>
fix budget 2022 nonglinshui
</commit_message>
<xml_diff>
--- a/data-raw/data-tidy/nation-yearbook/part07-finance/02-public-budget/2022.xlsx
+++ b/data-raw/data-tidy/nation-yearbook/part07-finance/02-public-budget/2022.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
   <si>
     <t xml:space="preserve">province</t>
   </si>
@@ -150,6 +150,12 @@
   </si>
   <si>
     <t xml:space="preserve">v6_cz_yszc_kxjs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">农林水</t>
+  </si>
+  <si>
+    <t xml:space="preserve">v6_cz_yszc_nls</t>
   </si>
 </sst>
 </file>
@@ -2418,6 +2424,646 @@
         <v>45</v>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" t="s">
+        <v>6</v>
+      </c>
+      <c r="B98" t="s">
+        <v>7</v>
+      </c>
+      <c r="C98" t="s">
+        <v>46</v>
+      </c>
+      <c r="D98" t="n">
+        <v>22250.21</v>
+      </c>
+      <c r="E98" t="s">
+        <v>9</v>
+      </c>
+      <c r="F98" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="s">
+        <v>11</v>
+      </c>
+      <c r="B99" t="s">
+        <v>7</v>
+      </c>
+      <c r="C99" t="s">
+        <v>46</v>
+      </c>
+      <c r="D99" t="n">
+        <v>462.79</v>
+      </c>
+      <c r="E99" t="s">
+        <v>9</v>
+      </c>
+      <c r="F99" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="s">
+        <v>12</v>
+      </c>
+      <c r="B100" t="s">
+        <v>7</v>
+      </c>
+      <c r="C100" t="s">
+        <v>46</v>
+      </c>
+      <c r="D100" t="n">
+        <v>110.3</v>
+      </c>
+      <c r="E100" t="s">
+        <v>9</v>
+      </c>
+      <c r="F100" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="s">
+        <v>13</v>
+      </c>
+      <c r="B101" t="s">
+        <v>7</v>
+      </c>
+      <c r="C101" t="s">
+        <v>46</v>
+      </c>
+      <c r="D101" t="n">
+        <v>872.14</v>
+      </c>
+      <c r="E101" t="s">
+        <v>9</v>
+      </c>
+      <c r="F101" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="s">
+        <v>14</v>
+      </c>
+      <c r="B102" t="s">
+        <v>7</v>
+      </c>
+      <c r="C102" t="s">
+        <v>46</v>
+      </c>
+      <c r="D102" t="n">
+        <v>576.87</v>
+      </c>
+      <c r="E102" t="s">
+        <v>9</v>
+      </c>
+      <c r="F102" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="s">
+        <v>15</v>
+      </c>
+      <c r="B103" t="s">
+        <v>7</v>
+      </c>
+      <c r="C103" t="s">
+        <v>46</v>
+      </c>
+      <c r="D103" t="n">
+        <v>912.44</v>
+      </c>
+      <c r="E103" t="s">
+        <v>9</v>
+      </c>
+      <c r="F103" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="s">
+        <v>16</v>
+      </c>
+      <c r="B104" t="s">
+        <v>7</v>
+      </c>
+      <c r="C104" t="s">
+        <v>46</v>
+      </c>
+      <c r="D104" t="n">
+        <v>463.34</v>
+      </c>
+      <c r="E104" t="s">
+        <v>9</v>
+      </c>
+      <c r="F104" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="s">
+        <v>17</v>
+      </c>
+      <c r="B105" t="s">
+        <v>7</v>
+      </c>
+      <c r="C105" t="s">
+        <v>46</v>
+      </c>
+      <c r="D105" t="n">
+        <v>515.49</v>
+      </c>
+      <c r="E105" t="s">
+        <v>9</v>
+      </c>
+      <c r="F105" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="s">
+        <v>18</v>
+      </c>
+      <c r="B106" t="s">
+        <v>7</v>
+      </c>
+      <c r="C106" t="s">
+        <v>46</v>
+      </c>
+      <c r="D106" t="n">
+        <v>937.59</v>
+      </c>
+      <c r="E106" t="s">
+        <v>9</v>
+      </c>
+      <c r="F106" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="s">
+        <v>19</v>
+      </c>
+      <c r="B107" t="s">
+        <v>7</v>
+      </c>
+      <c r="C107" t="s">
+        <v>46</v>
+      </c>
+      <c r="D107" t="n">
+        <v>388.62</v>
+      </c>
+      <c r="E107" t="s">
+        <v>9</v>
+      </c>
+      <c r="F107" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="s">
+        <v>20</v>
+      </c>
+      <c r="B108" t="s">
+        <v>7</v>
+      </c>
+      <c r="C108" t="s">
+        <v>46</v>
+      </c>
+      <c r="D108" t="n">
+        <v>1108.36</v>
+      </c>
+      <c r="E108" t="s">
+        <v>9</v>
+      </c>
+      <c r="F108" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="s">
+        <v>21</v>
+      </c>
+      <c r="B109" t="s">
+        <v>7</v>
+      </c>
+      <c r="C109" t="s">
+        <v>46</v>
+      </c>
+      <c r="D109" t="n">
+        <v>831.2</v>
+      </c>
+      <c r="E109" t="s">
+        <v>9</v>
+      </c>
+      <c r="F109" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="s">
+        <v>22</v>
+      </c>
+      <c r="B110" t="s">
+        <v>7</v>
+      </c>
+      <c r="C110" t="s">
+        <v>46</v>
+      </c>
+      <c r="D110" t="n">
+        <v>991.88</v>
+      </c>
+      <c r="E110" t="s">
+        <v>9</v>
+      </c>
+      <c r="F110" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="s">
+        <v>23</v>
+      </c>
+      <c r="B111" t="s">
+        <v>7</v>
+      </c>
+      <c r="C111" t="s">
+        <v>46</v>
+      </c>
+      <c r="D111" t="n">
+        <v>410.37</v>
+      </c>
+      <c r="E111" t="s">
+        <v>9</v>
+      </c>
+      <c r="F111" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="s">
+        <v>24</v>
+      </c>
+      <c r="B112" t="s">
+        <v>7</v>
+      </c>
+      <c r="C112" t="s">
+        <v>46</v>
+      </c>
+      <c r="D112" t="n">
+        <v>788.48</v>
+      </c>
+      <c r="E112" t="s">
+        <v>9</v>
+      </c>
+      <c r="F112" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="s">
+        <v>25</v>
+      </c>
+      <c r="B113" t="s">
+        <v>7</v>
+      </c>
+      <c r="C113" t="s">
+        <v>46</v>
+      </c>
+      <c r="D113" t="n">
+        <v>1118.86</v>
+      </c>
+      <c r="E113" t="s">
+        <v>9</v>
+      </c>
+      <c r="F113" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="s">
+        <v>26</v>
+      </c>
+      <c r="B114" t="s">
+        <v>7</v>
+      </c>
+      <c r="C114" t="s">
+        <v>46</v>
+      </c>
+      <c r="D114" t="n">
+        <v>1110.48</v>
+      </c>
+      <c r="E114" t="s">
+        <v>9</v>
+      </c>
+      <c r="F114" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="s">
+        <v>27</v>
+      </c>
+      <c r="B115" t="s">
+        <v>7</v>
+      </c>
+      <c r="C115" t="s">
+        <v>46</v>
+      </c>
+      <c r="D115" t="n">
+        <v>924.84</v>
+      </c>
+      <c r="E115" t="s">
+        <v>9</v>
+      </c>
+      <c r="F115" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="s">
+        <v>28</v>
+      </c>
+      <c r="B116" t="s">
+        <v>7</v>
+      </c>
+      <c r="C116" t="s">
+        <v>46</v>
+      </c>
+      <c r="D116" t="n">
+        <v>995.44</v>
+      </c>
+      <c r="E116" t="s">
+        <v>9</v>
+      </c>
+      <c r="F116" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="s">
+        <v>29</v>
+      </c>
+      <c r="B117" t="s">
+        <v>7</v>
+      </c>
+      <c r="C117" t="s">
+        <v>46</v>
+      </c>
+      <c r="D117" t="n">
+        <v>1067.57</v>
+      </c>
+      <c r="E117" t="s">
+        <v>9</v>
+      </c>
+      <c r="F117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="s">
+        <v>30</v>
+      </c>
+      <c r="B118" t="s">
+        <v>7</v>
+      </c>
+      <c r="C118" t="s">
+        <v>46</v>
+      </c>
+      <c r="D118" t="n">
+        <v>737.07</v>
+      </c>
+      <c r="E118" t="s">
+        <v>9</v>
+      </c>
+      <c r="F118" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="s">
+        <v>31</v>
+      </c>
+      <c r="B119" t="s">
+        <v>7</v>
+      </c>
+      <c r="C119" t="s">
+        <v>46</v>
+      </c>
+      <c r="D119" t="n">
+        <v>265.65</v>
+      </c>
+      <c r="E119" t="s">
+        <v>9</v>
+      </c>
+      <c r="F119" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="s">
+        <v>32</v>
+      </c>
+      <c r="B120" t="s">
+        <v>7</v>
+      </c>
+      <c r="C120" t="s">
+        <v>46</v>
+      </c>
+      <c r="D120" t="n">
+        <v>393.85</v>
+      </c>
+      <c r="E120" t="s">
+        <v>9</v>
+      </c>
+      <c r="F120" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="s">
+        <v>33</v>
+      </c>
+      <c r="B121" t="s">
+        <v>7</v>
+      </c>
+      <c r="C121" t="s">
+        <v>46</v>
+      </c>
+      <c r="D121" t="n">
+        <v>1359.32</v>
+      </c>
+      <c r="E121" t="s">
+        <v>9</v>
+      </c>
+      <c r="F121" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="s">
+        <v>34</v>
+      </c>
+      <c r="B122" t="s">
+        <v>7</v>
+      </c>
+      <c r="C122" t="s">
+        <v>46</v>
+      </c>
+      <c r="D122" t="n">
+        <v>692.15</v>
+      </c>
+      <c r="E122" t="s">
+        <v>9</v>
+      </c>
+      <c r="F122" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="s">
+        <v>35</v>
+      </c>
+      <c r="B123" t="s">
+        <v>7</v>
+      </c>
+      <c r="C123" t="s">
+        <v>46</v>
+      </c>
+      <c r="D123" t="n">
+        <v>888.43</v>
+      </c>
+      <c r="E123" t="s">
+        <v>9</v>
+      </c>
+      <c r="F123" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="s">
+        <v>36</v>
+      </c>
+      <c r="B124" t="s">
+        <v>7</v>
+      </c>
+      <c r="C124" t="s">
+        <v>46</v>
+      </c>
+      <c r="D124" t="n">
+        <v>371.87</v>
+      </c>
+      <c r="E124" t="s">
+        <v>9</v>
+      </c>
+      <c r="F124" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="s">
+        <v>37</v>
+      </c>
+      <c r="B125" t="s">
+        <v>7</v>
+      </c>
+      <c r="C125" t="s">
+        <v>46</v>
+      </c>
+      <c r="D125" t="n">
+        <v>733.21</v>
+      </c>
+      <c r="E125" t="s">
+        <v>9</v>
+      </c>
+      <c r="F125" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="s">
+        <v>38</v>
+      </c>
+      <c r="B126" t="s">
+        <v>7</v>
+      </c>
+      <c r="C126" t="s">
+        <v>46</v>
+      </c>
+      <c r="D126" t="n">
+        <v>751.51</v>
+      </c>
+      <c r="E126" t="s">
+        <v>9</v>
+      </c>
+      <c r="F126" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="s">
+        <v>39</v>
+      </c>
+      <c r="B127" t="s">
+        <v>7</v>
+      </c>
+      <c r="C127" t="s">
+        <v>46</v>
+      </c>
+      <c r="D127" t="n">
+        <v>275.13</v>
+      </c>
+      <c r="E127" t="s">
+        <v>9</v>
+      </c>
+      <c r="F127" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="s">
+        <v>40</v>
+      </c>
+      <c r="B128" t="s">
+        <v>7</v>
+      </c>
+      <c r="C128" t="s">
+        <v>46</v>
+      </c>
+      <c r="D128" t="n">
+        <v>244.88</v>
+      </c>
+      <c r="E128" t="s">
+        <v>9</v>
+      </c>
+      <c r="F128" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="s">
+        <v>41</v>
+      </c>
+      <c r="B129" t="s">
+        <v>7</v>
+      </c>
+      <c r="C129" t="s">
+        <v>46</v>
+      </c>
+      <c r="D129" t="n">
+        <v>950.09</v>
+      </c>
+      <c r="E129" t="s">
+        <v>9</v>
+      </c>
+      <c r="F129" t="s">
+        <v>47</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>